<commit_message>
feat: add manual detection review components and custom starry button styles
</commit_message>
<xml_diff>
--- a/excel/Tally.xlsx
+++ b/excel/Tally.xlsx
@@ -8179,13 +8179,13 @@
         <v>71</v>
       </c>
       <c r="B73" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C73" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D73" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E73" s="5" t="n">
         <v>5</v>
@@ -8194,37 +8194,37 @@
         <v>4</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H73" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I73" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J73" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K73" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L73" s="5" t="n">
         <v>3</v>
       </c>
       <c r="M73" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N73" s="5" t="n">
         <v>5</v>
       </c>
       <c r="O73" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P73" s="5" t="n">
         <v>4</v>
       </c>
       <c r="Q73" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R73" s="5" t="n">
         <v>4</v>
@@ -8236,37 +8236,37 @@
         <v>4</v>
       </c>
       <c r="U73" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V73" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W73" s="5" t="n">
         <v>3</v>
       </c>
       <c r="X73" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y73" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Z73" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AA73" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AB73" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC73" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AD73" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE73" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AF73" s="5" t="n">
         <v>4</v>

</xml_diff>